<commit_message>
pagina inicial desenvolvida Imagens adicionadas medidas atualizadas
</commit_message>
<xml_diff>
--- a/PDA_Competências.xlsx
+++ b/PDA_Competências.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6158ddbae350e453/Projetos VS Code/Verena/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{E4DD8B47-0049-43C6-AD19-DEB84C1C668F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A984FDF6-B6A8-4545-85AB-1380DFE26497}"/>
+  <xr:revisionPtr revIDLastSave="16" documentId="13_ncr:1_{E4DD8B47-0049-43C6-AD19-DEB84C1C668F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7903BE24-C0D8-4BD0-B992-3F77E73985DD}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{A46958BD-7D9E-4CA0-A73D-571F27924EC9}"/>
+    <workbookView xWindow="225" yWindow="5325" windowWidth="38175" windowHeight="15555" xr2:uid="{A46958BD-7D9E-4CA0-A73D-571F27924EC9}"/>
   </bookViews>
   <sheets>
     <sheet name="PDA" sheetId="2" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="103">
   <si>
     <t>Comunicação</t>
   </si>
@@ -258,13 +258,85 @@
   </si>
   <si>
     <t>filial</t>
+  </si>
+  <si>
+    <t>Ana Souza</t>
+  </si>
+  <si>
+    <t>Bruno Lima</t>
+  </si>
+  <si>
+    <t>Carla Mendes</t>
+  </si>
+  <si>
+    <t>Diego Ferreira</t>
+  </si>
+  <si>
+    <t>Eduarda Castro</t>
+  </si>
+  <si>
+    <t>Felipe Rocha</t>
+  </si>
+  <si>
+    <t>Gabriela Nunes</t>
+  </si>
+  <si>
+    <t>Henrique Souza</t>
+  </si>
+  <si>
+    <t>Isabela Tavares</t>
+  </si>
+  <si>
+    <t>Joao Pedro Alves</t>
+  </si>
+  <si>
+    <t>Camila</t>
+  </si>
+  <si>
+    <t>Gerente de Vendas</t>
+  </si>
+  <si>
+    <t>Supervisor de Linha</t>
+  </si>
+  <si>
+    <t>Analista de RH</t>
+  </si>
+  <si>
+    <t>Desenvolvedor</t>
+  </si>
+  <si>
+    <t>Vendedora</t>
+  </si>
+  <si>
+    <t>Analista Financeiro</t>
+  </si>
+  <si>
+    <t>Coordenadora de Marketing</t>
+  </si>
+  <si>
+    <t>Coordenador de Logistica</t>
+  </si>
+  <si>
+    <t>Atendente</t>
+  </si>
+  <si>
+    <t>Gerente de RH</t>
+  </si>
+  <si>
+    <t>Analista de TI</t>
+  </si>
+  <si>
+    <t>Pouco_consistente</t>
+  </si>
+  <si>
+    <t>Inválido</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="19">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -395,6 +467,14 @@
     <font>
       <sz val="11"/>
       <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -821,7 +901,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
@@ -867,6 +947,7 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Ênfase1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1242,15 +1323,37 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D94B368E-268C-4F99-99E6-8D1A085E8388}">
-  <dimension ref="A1:AH6"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:AH17"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="2.21875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="22.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.77734375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="2.875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.25" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="30.25" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.75" bestFit="1" customWidth="1"/>
+    <col min="6" max="8" width="8.625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="8.5" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.375" bestFit="1" customWidth="1"/>
+    <col min="11" max="13" width="11.25" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="11.125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="10.75" bestFit="1" customWidth="1"/>
+    <col min="16" max="18" width="10.625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="13.5" bestFit="1" customWidth="1"/>
+    <col min="21" max="23" width="13.375" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="13.25" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="9.875" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="9.875" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="3.375" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="3.5" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="11.5" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.875" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="11" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="11.875" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="3.125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:34" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:34">
       <c r="A1" t="s">
         <v>68</v>
       </c>
@@ -1354,7 +1457,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="2" spans="1:34" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:34">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1458,7 +1561,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="3" spans="1:34" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:34">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1562,7 +1665,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:34" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:34">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1666,7 +1769,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:34" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:34">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1770,7 +1873,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="6" spans="1:34" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:34">
       <c r="A6">
         <v>5</v>
       </c>
@@ -1872,23 +1975,1168 @@
       </c>
       <c r="AH6">
         <v>11</v>
+      </c>
+    </row>
+    <row r="7" spans="1:34">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>79</v>
+      </c>
+      <c r="C7" t="s">
+        <v>69</v>
+      </c>
+      <c r="D7" t="s">
+        <v>90</v>
+      </c>
+      <c r="E7">
+        <v>85</v>
+      </c>
+      <c r="F7">
+        <v>90</v>
+      </c>
+      <c r="G7">
+        <v>15</v>
+      </c>
+      <c r="H7">
+        <v>10</v>
+      </c>
+      <c r="I7">
+        <v>55</v>
+      </c>
+      <c r="J7">
+        <v>78</v>
+      </c>
+      <c r="K7">
+        <v>82</v>
+      </c>
+      <c r="L7">
+        <v>30</v>
+      </c>
+      <c r="M7">
+        <v>25</v>
+      </c>
+      <c r="N7">
+        <v>52</v>
+      </c>
+      <c r="O7">
+        <v>75</v>
+      </c>
+      <c r="P7">
+        <v>80</v>
+      </c>
+      <c r="Q7">
+        <v>25</v>
+      </c>
+      <c r="R7">
+        <v>20</v>
+      </c>
+      <c r="S7">
+        <v>60</v>
+      </c>
+      <c r="T7">
+        <v>70</v>
+      </c>
+      <c r="U7">
+        <v>75</v>
+      </c>
+      <c r="V7">
+        <v>35</v>
+      </c>
+      <c r="W7">
+        <v>30</v>
+      </c>
+      <c r="X7">
+        <v>55</v>
+      </c>
+      <c r="Y7">
+        <v>88</v>
+      </c>
+      <c r="Z7">
+        <v>72</v>
+      </c>
+      <c r="AA7">
+        <v>65</v>
+      </c>
+      <c r="AB7">
+        <v>55</v>
+      </c>
+      <c r="AC7">
+        <v>45</v>
+      </c>
+      <c r="AD7" t="s">
+        <v>76</v>
+      </c>
+      <c r="AE7">
+        <v>84</v>
+      </c>
+      <c r="AF7">
+        <v>91</v>
+      </c>
+      <c r="AG7">
+        <v>62</v>
+      </c>
+      <c r="AH7" s="19">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="8" spans="1:34">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>80</v>
+      </c>
+      <c r="C8" t="s">
+        <v>70</v>
+      </c>
+      <c r="D8" t="s">
+        <v>91</v>
+      </c>
+      <c r="E8">
+        <v>30</v>
+      </c>
+      <c r="F8">
+        <v>20</v>
+      </c>
+      <c r="G8">
+        <v>80</v>
+      </c>
+      <c r="H8">
+        <v>70</v>
+      </c>
+      <c r="I8">
+        <v>75</v>
+      </c>
+      <c r="J8">
+        <v>28</v>
+      </c>
+      <c r="K8">
+        <v>18</v>
+      </c>
+      <c r="L8">
+        <v>72</v>
+      </c>
+      <c r="M8">
+        <v>68</v>
+      </c>
+      <c r="N8">
+        <v>80</v>
+      </c>
+      <c r="O8">
+        <v>15</v>
+      </c>
+      <c r="P8">
+        <v>30</v>
+      </c>
+      <c r="Q8">
+        <v>75</v>
+      </c>
+      <c r="R8">
+        <v>80</v>
+      </c>
+      <c r="S8">
+        <v>65</v>
+      </c>
+      <c r="T8">
+        <v>18</v>
+      </c>
+      <c r="U8">
+        <v>25</v>
+      </c>
+      <c r="V8">
+        <v>70</v>
+      </c>
+      <c r="W8">
+        <v>76</v>
+      </c>
+      <c r="X8">
+        <v>62</v>
+      </c>
+      <c r="Y8">
+        <v>18</v>
+      </c>
+      <c r="Z8">
+        <v>58</v>
+      </c>
+      <c r="AA8">
+        <v>38</v>
+      </c>
+      <c r="AB8">
+        <v>68</v>
+      </c>
+      <c r="AC8">
+        <v>72</v>
+      </c>
+      <c r="AD8" t="s">
+        <v>76</v>
+      </c>
+      <c r="AE8">
+        <v>93</v>
+      </c>
+      <c r="AF8">
+        <v>52</v>
+      </c>
+      <c r="AG8">
+        <v>66</v>
+      </c>
+      <c r="AH8" s="19">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="9" spans="1:34">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
+        <v>81</v>
+      </c>
+      <c r="C9" t="s">
+        <v>70</v>
+      </c>
+      <c r="D9" t="s">
+        <v>92</v>
+      </c>
+      <c r="E9">
+        <v>20</v>
+      </c>
+      <c r="F9">
+        <v>75</v>
+      </c>
+      <c r="G9">
+        <v>65</v>
+      </c>
+      <c r="H9">
+        <v>40</v>
+      </c>
+      <c r="I9">
+        <v>30</v>
+      </c>
+      <c r="J9">
+        <v>15</v>
+      </c>
+      <c r="K9">
+        <v>72</v>
+      </c>
+      <c r="L9">
+        <v>60</v>
+      </c>
+      <c r="M9">
+        <v>38</v>
+      </c>
+      <c r="N9">
+        <v>28</v>
+      </c>
+      <c r="O9">
+        <v>30</v>
+      </c>
+      <c r="P9">
+        <v>65</v>
+      </c>
+      <c r="Q9">
+        <v>60</v>
+      </c>
+      <c r="R9">
+        <v>45</v>
+      </c>
+      <c r="S9">
+        <v>35</v>
+      </c>
+      <c r="T9">
+        <v>18</v>
+      </c>
+      <c r="U9">
+        <v>62</v>
+      </c>
+      <c r="V9">
+        <v>58</v>
+      </c>
+      <c r="W9">
+        <v>40</v>
+      </c>
+      <c r="X9">
+        <v>32</v>
+      </c>
+      <c r="Y9">
+        <v>42</v>
+      </c>
+      <c r="Z9">
+        <v>55</v>
+      </c>
+      <c r="AA9">
+        <v>42</v>
+      </c>
+      <c r="AB9">
+        <v>40</v>
+      </c>
+      <c r="AC9">
+        <v>75</v>
+      </c>
+      <c r="AD9" t="s">
+        <v>76</v>
+      </c>
+      <c r="AE9">
+        <v>73</v>
+      </c>
+      <c r="AF9">
+        <v>56</v>
+      </c>
+      <c r="AG9">
+        <v>72</v>
+      </c>
+      <c r="AH9" s="19">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="10" spans="1:34">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>82</v>
+      </c>
+      <c r="C10" t="s">
+        <v>70</v>
+      </c>
+      <c r="D10" t="s">
+        <v>93</v>
+      </c>
+      <c r="E10">
+        <v>40</v>
+      </c>
+      <c r="F10">
+        <v>15</v>
+      </c>
+      <c r="G10">
+        <v>55</v>
+      </c>
+      <c r="H10">
+        <v>90</v>
+      </c>
+      <c r="I10">
+        <v>85</v>
+      </c>
+      <c r="J10">
+        <v>38</v>
+      </c>
+      <c r="K10">
+        <v>12</v>
+      </c>
+      <c r="L10">
+        <v>52</v>
+      </c>
+      <c r="M10">
+        <v>82</v>
+      </c>
+      <c r="N10">
+        <v>80</v>
+      </c>
+      <c r="O10">
+        <v>45</v>
+      </c>
+      <c r="P10">
+        <v>25</v>
+      </c>
+      <c r="Q10">
+        <v>50</v>
+      </c>
+      <c r="R10">
+        <v>85</v>
+      </c>
+      <c r="S10">
+        <v>80</v>
+      </c>
+      <c r="T10">
+        <v>40</v>
+      </c>
+      <c r="U10">
+        <v>18</v>
+      </c>
+      <c r="V10">
+        <v>48</v>
+      </c>
+      <c r="W10">
+        <v>80</v>
+      </c>
+      <c r="X10">
+        <v>78</v>
+      </c>
+      <c r="Y10">
+        <v>38</v>
+      </c>
+      <c r="Z10">
+        <v>62</v>
+      </c>
+      <c r="AA10">
+        <v>45</v>
+      </c>
+      <c r="AB10">
+        <v>52</v>
+      </c>
+      <c r="AC10">
+        <v>80</v>
+      </c>
+      <c r="AD10" t="s">
+        <v>76</v>
+      </c>
+      <c r="AE10">
+        <v>70</v>
+      </c>
+      <c r="AF10">
+        <v>62</v>
+      </c>
+      <c r="AG10">
+        <v>73</v>
+      </c>
+      <c r="AH10" s="19">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="11" spans="1:34">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
+        <v>83</v>
+      </c>
+      <c r="C11" t="s">
+        <v>70</v>
+      </c>
+      <c r="D11" t="s">
+        <v>94</v>
+      </c>
+      <c r="E11">
+        <v>75</v>
+      </c>
+      <c r="F11">
+        <v>95</v>
+      </c>
+      <c r="G11">
+        <v>30</v>
+      </c>
+      <c r="H11">
+        <v>0</v>
+      </c>
+      <c r="I11">
+        <v>20</v>
+      </c>
+      <c r="J11">
+        <v>70</v>
+      </c>
+      <c r="K11">
+        <v>92</v>
+      </c>
+      <c r="L11">
+        <v>28</v>
+      </c>
+      <c r="M11">
+        <v>8</v>
+      </c>
+      <c r="N11">
+        <v>18</v>
+      </c>
+      <c r="O11">
+        <v>70</v>
+      </c>
+      <c r="P11">
+        <v>88</v>
+      </c>
+      <c r="Q11">
+        <v>35</v>
+      </c>
+      <c r="R11">
+        <v>7</v>
+      </c>
+      <c r="S11">
+        <v>28</v>
+      </c>
+      <c r="T11">
+        <v>68</v>
+      </c>
+      <c r="U11">
+        <v>85</v>
+      </c>
+      <c r="V11">
+        <v>32</v>
+      </c>
+      <c r="W11">
+        <v>12</v>
+      </c>
+      <c r="X11">
+        <v>25</v>
+      </c>
+      <c r="Y11">
+        <v>84</v>
+      </c>
+      <c r="Z11">
+        <v>78</v>
+      </c>
+      <c r="AA11">
+        <v>70</v>
+      </c>
+      <c r="AB11">
+        <v>48</v>
+      </c>
+      <c r="AC11">
+        <v>68</v>
+      </c>
+      <c r="AD11" t="s">
+        <v>76</v>
+      </c>
+      <c r="AE11">
+        <v>81</v>
+      </c>
+      <c r="AF11">
+        <v>74</v>
+      </c>
+      <c r="AG11">
+        <v>60</v>
+      </c>
+      <c r="AH11" s="19">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="12" spans="1:34">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" t="s">
+        <v>84</v>
+      </c>
+      <c r="C12" t="s">
+        <v>69</v>
+      </c>
+      <c r="D12" t="s">
+        <v>95</v>
+      </c>
+      <c r="E12">
+        <v>25</v>
+      </c>
+      <c r="F12">
+        <v>30</v>
+      </c>
+      <c r="G12">
+        <v>70</v>
+      </c>
+      <c r="H12">
+        <v>75</v>
+      </c>
+      <c r="I12">
+        <v>90</v>
+      </c>
+      <c r="J12">
+        <v>22</v>
+      </c>
+      <c r="K12">
+        <v>28</v>
+      </c>
+      <c r="L12">
+        <v>68</v>
+      </c>
+      <c r="M12">
+        <v>72</v>
+      </c>
+      <c r="N12">
+        <v>88</v>
+      </c>
+      <c r="O12">
+        <v>30</v>
+      </c>
+      <c r="P12">
+        <v>35</v>
+      </c>
+      <c r="Q12">
+        <v>65</v>
+      </c>
+      <c r="R12">
+        <v>70</v>
+      </c>
+      <c r="S12">
+        <v>85</v>
+      </c>
+      <c r="T12">
+        <v>28</v>
+      </c>
+      <c r="U12">
+        <v>32</v>
+      </c>
+      <c r="V12">
+        <v>60</v>
+      </c>
+      <c r="W12">
+        <v>68</v>
+      </c>
+      <c r="X12">
+        <v>82</v>
+      </c>
+      <c r="Y12">
+        <v>40</v>
+      </c>
+      <c r="Z12">
+        <v>48</v>
+      </c>
+      <c r="AA12">
+        <v>35</v>
+      </c>
+      <c r="AB12">
+        <v>58</v>
+      </c>
+      <c r="AC12">
+        <v>80</v>
+      </c>
+      <c r="AD12" t="s">
+        <v>76</v>
+      </c>
+      <c r="AE12">
+        <v>61</v>
+      </c>
+      <c r="AF12">
+        <v>71</v>
+      </c>
+      <c r="AG12">
+        <v>81</v>
+      </c>
+      <c r="AH12" s="19">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="13" spans="1:34">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" t="s">
+        <v>85</v>
+      </c>
+      <c r="C13" t="s">
+        <v>70</v>
+      </c>
+      <c r="D13" t="s">
+        <v>96</v>
+      </c>
+      <c r="E13">
+        <v>55</v>
+      </c>
+      <c r="F13">
+        <v>85</v>
+      </c>
+      <c r="G13">
+        <v>45</v>
+      </c>
+      <c r="H13">
+        <v>15</v>
+      </c>
+      <c r="I13">
+        <v>40</v>
+      </c>
+      <c r="J13">
+        <v>50</v>
+      </c>
+      <c r="K13">
+        <v>80</v>
+      </c>
+      <c r="L13">
+        <v>42</v>
+      </c>
+      <c r="M13">
+        <v>12</v>
+      </c>
+      <c r="N13">
+        <v>38</v>
+      </c>
+      <c r="O13">
+        <v>60</v>
+      </c>
+      <c r="P13">
+        <v>80</v>
+      </c>
+      <c r="Q13">
+        <v>40</v>
+      </c>
+      <c r="R13">
+        <v>20</v>
+      </c>
+      <c r="S13">
+        <v>45</v>
+      </c>
+      <c r="T13">
+        <v>55</v>
+      </c>
+      <c r="U13">
+        <v>76</v>
+      </c>
+      <c r="V13">
+        <v>38</v>
+      </c>
+      <c r="W13">
+        <v>18</v>
+      </c>
+      <c r="X13">
+        <v>42</v>
+      </c>
+      <c r="Y13">
+        <v>72</v>
+      </c>
+      <c r="Z13">
+        <v>62</v>
+      </c>
+      <c r="AA13">
+        <v>55</v>
+      </c>
+      <c r="AB13">
+        <v>50</v>
+      </c>
+      <c r="AC13">
+        <v>65</v>
+      </c>
+      <c r="AD13" t="s">
+        <v>101</v>
+      </c>
+      <c r="AE13">
+        <v>82</v>
+      </c>
+      <c r="AF13">
+        <v>89</v>
+      </c>
+      <c r="AG13">
+        <v>89</v>
+      </c>
+      <c r="AH13" s="19">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="14" spans="1:34">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" t="s">
+        <v>86</v>
+      </c>
+      <c r="C14" t="s">
+        <v>70</v>
+      </c>
+      <c r="D14" t="s">
+        <v>97</v>
+      </c>
+      <c r="E14">
+        <v>90</v>
+      </c>
+      <c r="F14">
+        <v>40</v>
+      </c>
+      <c r="G14">
+        <v>10</v>
+      </c>
+      <c r="H14">
+        <v>60</v>
+      </c>
+      <c r="I14">
+        <v>65</v>
+      </c>
+      <c r="J14">
+        <v>85</v>
+      </c>
+      <c r="K14">
+        <v>38</v>
+      </c>
+      <c r="L14">
+        <v>8</v>
+      </c>
+      <c r="M14">
+        <v>55</v>
+      </c>
+      <c r="N14">
+        <v>62</v>
+      </c>
+      <c r="O14">
+        <v>80</v>
+      </c>
+      <c r="P14">
+        <v>45</v>
+      </c>
+      <c r="Q14">
+        <v>20</v>
+      </c>
+      <c r="R14">
+        <v>65</v>
+      </c>
+      <c r="S14">
+        <v>60</v>
+      </c>
+      <c r="T14">
+        <v>76</v>
+      </c>
+      <c r="U14">
+        <v>42</v>
+      </c>
+      <c r="V14">
+        <v>18</v>
+      </c>
+      <c r="W14">
+        <v>60</v>
+      </c>
+      <c r="X14">
+        <v>58</v>
+      </c>
+      <c r="Y14">
+        <v>80</v>
+      </c>
+      <c r="Z14">
+        <v>68</v>
+      </c>
+      <c r="AA14">
+        <v>75</v>
+      </c>
+      <c r="AB14">
+        <v>40</v>
+      </c>
+      <c r="AC14">
+        <v>72</v>
+      </c>
+      <c r="AD14" t="s">
+        <v>76</v>
+      </c>
+      <c r="AE14">
+        <v>75</v>
+      </c>
+      <c r="AF14">
+        <v>61</v>
+      </c>
+      <c r="AG14">
+        <v>75</v>
+      </c>
+      <c r="AH14" s="19">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="15" spans="1:34">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" t="s">
+        <v>87</v>
+      </c>
+      <c r="C15" t="s">
+        <v>70</v>
+      </c>
+      <c r="D15" t="s">
+        <v>98</v>
+      </c>
+      <c r="E15">
+        <v>15</v>
+      </c>
+      <c r="F15">
+        <v>80</v>
+      </c>
+      <c r="G15">
+        <v>70</v>
+      </c>
+      <c r="H15">
+        <v>35</v>
+      </c>
+      <c r="I15">
+        <v>25</v>
+      </c>
+      <c r="J15">
+        <v>12</v>
+      </c>
+      <c r="K15">
+        <v>76</v>
+      </c>
+      <c r="L15">
+        <v>65</v>
+      </c>
+      <c r="M15">
+        <v>32</v>
+      </c>
+      <c r="N15">
+        <v>22</v>
+      </c>
+      <c r="O15">
+        <v>25</v>
+      </c>
+      <c r="P15">
+        <v>70</v>
+      </c>
+      <c r="Q15">
+        <v>60</v>
+      </c>
+      <c r="R15">
+        <v>40</v>
+      </c>
+      <c r="S15">
+        <v>30</v>
+      </c>
+      <c r="T15">
+        <v>20</v>
+      </c>
+      <c r="U15">
+        <v>65</v>
+      </c>
+      <c r="V15">
+        <v>55</v>
+      </c>
+      <c r="W15">
+        <v>38</v>
+      </c>
+      <c r="X15">
+        <v>28</v>
+      </c>
+      <c r="Y15">
+        <v>30</v>
+      </c>
+      <c r="Z15">
+        <v>58</v>
+      </c>
+      <c r="AA15">
+        <v>38</v>
+      </c>
+      <c r="AB15">
+        <v>62</v>
+      </c>
+      <c r="AC15">
+        <v>82</v>
+      </c>
+      <c r="AD15" t="s">
+        <v>102</v>
+      </c>
+      <c r="AE15">
+        <v>73</v>
+      </c>
+      <c r="AF15">
+        <v>56</v>
+      </c>
+      <c r="AG15">
+        <v>89</v>
+      </c>
+      <c r="AH15" s="19">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="16" spans="1:34">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16" t="s">
+        <v>88</v>
+      </c>
+      <c r="C16" t="s">
+        <v>69</v>
+      </c>
+      <c r="D16" t="s">
+        <v>99</v>
+      </c>
+      <c r="E16">
+        <v>60</v>
+      </c>
+      <c r="F16">
+        <v>60</v>
+      </c>
+      <c r="G16">
+        <v>40</v>
+      </c>
+      <c r="H16">
+        <v>40</v>
+      </c>
+      <c r="I16">
+        <v>50</v>
+      </c>
+      <c r="J16">
+        <v>55</v>
+      </c>
+      <c r="K16">
+        <v>55</v>
+      </c>
+      <c r="L16">
+        <v>38</v>
+      </c>
+      <c r="M16">
+        <v>38</v>
+      </c>
+      <c r="N16">
+        <v>48</v>
+      </c>
+      <c r="O16">
+        <v>55</v>
+      </c>
+      <c r="P16">
+        <v>55</v>
+      </c>
+      <c r="Q16">
+        <v>42</v>
+      </c>
+      <c r="R16">
+        <v>48</v>
+      </c>
+      <c r="S16">
+        <v>52</v>
+      </c>
+      <c r="T16">
+        <v>50</v>
+      </c>
+      <c r="U16">
+        <v>52</v>
+      </c>
+      <c r="V16">
+        <v>40</v>
+      </c>
+      <c r="W16">
+        <v>45</v>
+      </c>
+      <c r="X16">
+        <v>50</v>
+      </c>
+      <c r="Y16">
+        <v>60</v>
+      </c>
+      <c r="Z16">
+        <v>52</v>
+      </c>
+      <c r="AA16">
+        <v>48</v>
+      </c>
+      <c r="AB16">
+        <v>45</v>
+      </c>
+      <c r="AC16">
+        <v>70</v>
+      </c>
+      <c r="AD16" t="s">
+        <v>76</v>
+      </c>
+      <c r="AE16">
+        <v>63</v>
+      </c>
+      <c r="AF16">
+        <v>67</v>
+      </c>
+      <c r="AG16">
+        <v>98</v>
+      </c>
+      <c r="AH16" s="19">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="17" spans="1:34">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17" t="s">
+        <v>89</v>
+      </c>
+      <c r="C17" t="s">
+        <v>70</v>
+      </c>
+      <c r="D17" t="s">
+        <v>100</v>
+      </c>
+      <c r="E17">
+        <v>100</v>
+      </c>
+      <c r="F17">
+        <v>50</v>
+      </c>
+      <c r="G17">
+        <v>8</v>
+      </c>
+      <c r="H17">
+        <v>42</v>
+      </c>
+      <c r="I17">
+        <v>4</v>
+      </c>
+      <c r="J17">
+        <v>69</v>
+      </c>
+      <c r="K17">
+        <v>50</v>
+      </c>
+      <c r="L17">
+        <v>36</v>
+      </c>
+      <c r="M17">
+        <v>48</v>
+      </c>
+      <c r="N17">
+        <v>36</v>
+      </c>
+      <c r="O17">
+        <v>100</v>
+      </c>
+      <c r="P17">
+        <v>42</v>
+      </c>
+      <c r="Q17">
+        <v>29</v>
+      </c>
+      <c r="R17">
+        <v>29</v>
+      </c>
+      <c r="S17">
+        <v>43</v>
+      </c>
+      <c r="T17">
+        <v>84</v>
+      </c>
+      <c r="U17">
+        <v>47</v>
+      </c>
+      <c r="V17">
+        <v>39</v>
+      </c>
+      <c r="W17">
+        <v>39</v>
+      </c>
+      <c r="X17">
+        <v>47</v>
+      </c>
+      <c r="Y17">
+        <v>82</v>
+      </c>
+      <c r="Z17">
+        <v>40</v>
+      </c>
+      <c r="AA17">
+        <v>27</v>
+      </c>
+      <c r="AB17">
+        <v>61</v>
+      </c>
+      <c r="AC17">
+        <v>80</v>
+      </c>
+      <c r="AD17" t="s">
+        <v>76</v>
+      </c>
+      <c r="AE17">
+        <v>59</v>
+      </c>
+      <c r="AF17">
+        <v>70</v>
+      </c>
+      <c r="AG17">
+        <v>57</v>
+      </c>
+      <c r="AH17" s="19">
+        <v>20</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0CB43BE2-CB00-4D75-B765-4304459626ED}">
   <dimension ref="A1:Z8"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="1.77734375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="22.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="1.75" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:26" ht="15">
       <c r="B1" s="9" t="s">
         <v>66</v>
       </c>
@@ -1923,7 +3171,7 @@
       <c r="Y1" s="14"/>
       <c r="Z1" s="15"/>
     </row>
-    <row r="2" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:26">
       <c r="B2" t="s">
         <v>64</v>
       </c>
@@ -1986,7 +3234,7 @@
       <c r="Y2" s="17"/>
       <c r="Z2" s="18"/>
     </row>
-    <row r="3" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:26">
       <c r="B3" t="s">
         <v>65</v>
       </c>
@@ -2047,7 +3295,7 @@
       <c r="Y3" s="17"/>
       <c r="Z3" s="18"/>
     </row>
-    <row r="4" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:26">
       <c r="A4">
         <v>1</v>
       </c>
@@ -2105,7 +3353,7 @@
       <c r="S4" s="1"/>
       <c r="Z4" s="2"/>
     </row>
-    <row r="5" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:26">
       <c r="A5">
         <v>2</v>
       </c>
@@ -2163,7 +3411,7 @@
       <c r="S5" s="1"/>
       <c r="Z5" s="2"/>
     </row>
-    <row r="6" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:26">
       <c r="A6">
         <v>3</v>
       </c>
@@ -2221,7 +3469,7 @@
       <c r="S6" s="1"/>
       <c r="Z6" s="2"/>
     </row>
-    <row r="7" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:26">
       <c r="A7">
         <v>4</v>
       </c>
@@ -2279,7 +3527,7 @@
       <c r="S7" s="1"/>
       <c r="Z7" s="2"/>
     </row>
-    <row r="8" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:26">
       <c r="A8">
         <v>5</v>
       </c>

</xml_diff>

<commit_message>
Perfil da empresa completo
</commit_message>
<xml_diff>
--- a/PDA_Competências.xlsx
+++ b/PDA_Competências.xlsx
@@ -8,20 +8,31 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6158ddbae350e453/Projetos VS Code/Verena/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="16" documentId="13_ncr:1_{E4DD8B47-0049-43C6-AD19-DEB84C1C668F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7903BE24-C0D8-4BD0-B992-3F77E73985DD}"/>
+  <xr:revisionPtr revIDLastSave="20" documentId="13_ncr:1_{E4DD8B47-0049-43C6-AD19-DEB84C1C668F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{62AB4F4C-61DD-4C21-A0E4-AB2DBF3DC319}"/>
   <bookViews>
-    <workbookView xWindow="225" yWindow="5325" windowWidth="38175" windowHeight="15555" xr2:uid="{A46958BD-7D9E-4CA0-A73D-571F27924EC9}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{A46958BD-7D9E-4CA0-A73D-571F27924EC9}"/>
   </bookViews>
   <sheets>
     <sheet name="PDA" sheetId="2" r:id="rId1"/>
     <sheet name="Competências" sheetId="1" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="95">
   <si>
     <t>Comunicação</t>
   </si>
@@ -300,30 +311,6 @@
   </si>
   <si>
     <t>Analista de RH</t>
-  </si>
-  <si>
-    <t>Desenvolvedor</t>
-  </si>
-  <si>
-    <t>Vendedora</t>
-  </si>
-  <si>
-    <t>Analista Financeiro</t>
-  </si>
-  <si>
-    <t>Coordenadora de Marketing</t>
-  </si>
-  <si>
-    <t>Coordenador de Logistica</t>
-  </si>
-  <si>
-    <t>Atendente</t>
-  </si>
-  <si>
-    <t>Gerente de RH</t>
-  </si>
-  <si>
-    <t>Analista de TI</t>
   </si>
   <si>
     <t>Pouco_consistente</t>
@@ -929,6 +916,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -947,7 +935,6 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Ênfase1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -2077,7 +2064,7 @@
       <c r="AG7">
         <v>62</v>
       </c>
-      <c r="AH7" s="19">
+      <c r="AH7" s="13">
         <v>20</v>
       </c>
     </row>
@@ -2092,7 +2079,7 @@
         <v>70</v>
       </c>
       <c r="D8" t="s">
-        <v>91</v>
+        <v>71</v>
       </c>
       <c r="E8">
         <v>30</v>
@@ -2181,7 +2168,7 @@
       <c r="AG8">
         <v>66</v>
       </c>
-      <c r="AH8" s="19">
+      <c r="AH8" s="13">
         <v>20</v>
       </c>
     </row>
@@ -2196,7 +2183,7 @@
         <v>70</v>
       </c>
       <c r="D9" t="s">
-        <v>92</v>
+        <v>72</v>
       </c>
       <c r="E9">
         <v>20</v>
@@ -2285,7 +2272,7 @@
       <c r="AG9">
         <v>72</v>
       </c>
-      <c r="AH9" s="19">
+      <c r="AH9" s="13">
         <v>20</v>
       </c>
     </row>
@@ -2300,7 +2287,7 @@
         <v>70</v>
       </c>
       <c r="D10" t="s">
-        <v>93</v>
+        <v>73</v>
       </c>
       <c r="E10">
         <v>40</v>
@@ -2389,7 +2376,7 @@
       <c r="AG10">
         <v>73</v>
       </c>
-      <c r="AH10" s="19">
+      <c r="AH10" s="13">
         <v>20</v>
       </c>
     </row>
@@ -2404,7 +2391,7 @@
         <v>70</v>
       </c>
       <c r="D11" t="s">
-        <v>94</v>
+        <v>74</v>
       </c>
       <c r="E11">
         <v>75</v>
@@ -2493,7 +2480,7 @@
       <c r="AG11">
         <v>60</v>
       </c>
-      <c r="AH11" s="19">
+      <c r="AH11" s="13">
         <v>20</v>
       </c>
     </row>
@@ -2508,7 +2495,7 @@
         <v>69</v>
       </c>
       <c r="D12" t="s">
-        <v>95</v>
+        <v>75</v>
       </c>
       <c r="E12">
         <v>25</v>
@@ -2597,7 +2584,7 @@
       <c r="AG12">
         <v>81</v>
       </c>
-      <c r="AH12" s="19">
+      <c r="AH12" s="13">
         <v>20</v>
       </c>
     </row>
@@ -2612,7 +2599,7 @@
         <v>70</v>
       </c>
       <c r="D13" t="s">
-        <v>96</v>
+        <v>90</v>
       </c>
       <c r="E13">
         <v>55</v>
@@ -2690,7 +2677,7 @@
         <v>65</v>
       </c>
       <c r="AD13" t="s">
-        <v>101</v>
+        <v>93</v>
       </c>
       <c r="AE13">
         <v>82</v>
@@ -2701,7 +2688,7 @@
       <c r="AG13">
         <v>89</v>
       </c>
-      <c r="AH13" s="19">
+      <c r="AH13" s="13">
         <v>20</v>
       </c>
     </row>
@@ -2716,7 +2703,7 @@
         <v>70</v>
       </c>
       <c r="D14" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="E14">
         <v>90</v>
@@ -2805,7 +2792,7 @@
       <c r="AG14">
         <v>75</v>
       </c>
-      <c r="AH14" s="19">
+      <c r="AH14" s="13">
         <v>20</v>
       </c>
     </row>
@@ -2820,7 +2807,7 @@
         <v>70</v>
       </c>
       <c r="D15" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="E15">
         <v>15</v>
@@ -2898,7 +2885,7 @@
         <v>82</v>
       </c>
       <c r="AD15" t="s">
-        <v>102</v>
+        <v>94</v>
       </c>
       <c r="AE15">
         <v>73</v>
@@ -2909,7 +2896,7 @@
       <c r="AG15">
         <v>89</v>
       </c>
-      <c r="AH15" s="19">
+      <c r="AH15" s="13">
         <v>20</v>
       </c>
     </row>
@@ -2924,7 +2911,7 @@
         <v>69</v>
       </c>
       <c r="D16" t="s">
-        <v>99</v>
+        <v>72</v>
       </c>
       <c r="E16">
         <v>60</v>
@@ -3013,7 +3000,7 @@
       <c r="AG16">
         <v>98</v>
       </c>
-      <c r="AH16" s="19">
+      <c r="AH16" s="13">
         <v>20</v>
       </c>
     </row>
@@ -3028,7 +3015,7 @@
         <v>70</v>
       </c>
       <c r="D17" t="s">
-        <v>100</v>
+        <v>73</v>
       </c>
       <c r="E17">
         <v>100</v>
@@ -3117,7 +3104,7 @@
       <c r="AG17">
         <v>57</v>
       </c>
-      <c r="AH17" s="19">
+      <c r="AH17" s="13">
         <v>20</v>
       </c>
     </row>
@@ -3140,36 +3127,36 @@
       <c r="B1" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="C1" s="13" t="s">
+      <c r="C1" s="14" t="s">
         <v>62</v>
       </c>
-      <c r="D1" s="14"/>
-      <c r="E1" s="14"/>
-      <c r="F1" s="14"/>
-      <c r="G1" s="14"/>
-      <c r="H1" s="14"/>
-      <c r="I1" s="14"/>
-      <c r="J1" s="15"/>
-      <c r="K1" s="13" t="s">
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
+      <c r="G1" s="15"/>
+      <c r="H1" s="15"/>
+      <c r="I1" s="15"/>
+      <c r="J1" s="16"/>
+      <c r="K1" s="14" t="s">
         <v>63</v>
       </c>
-      <c r="L1" s="14"/>
-      <c r="M1" s="14"/>
-      <c r="N1" s="14"/>
-      <c r="O1" s="14"/>
-      <c r="P1" s="14"/>
-      <c r="Q1" s="14"/>
-      <c r="R1" s="15"/>
-      <c r="S1" s="13" t="s">
+      <c r="L1" s="15"/>
+      <c r="M1" s="15"/>
+      <c r="N1" s="15"/>
+      <c r="O1" s="15"/>
+      <c r="P1" s="15"/>
+      <c r="Q1" s="15"/>
+      <c r="R1" s="16"/>
+      <c r="S1" s="14" t="s">
         <v>67</v>
       </c>
-      <c r="T1" s="14"/>
-      <c r="U1" s="14"/>
-      <c r="V1" s="14"/>
-      <c r="W1" s="14"/>
-      <c r="X1" s="14"/>
-      <c r="Y1" s="14"/>
-      <c r="Z1" s="15"/>
+      <c r="T1" s="15"/>
+      <c r="U1" s="15"/>
+      <c r="V1" s="15"/>
+      <c r="W1" s="15"/>
+      <c r="X1" s="15"/>
+      <c r="Y1" s="15"/>
+      <c r="Z1" s="16"/>
     </row>
     <row r="2" spans="1:26">
       <c r="B2" t="s">
@@ -3223,16 +3210,16 @@
       <c r="R2" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="S2" s="16" t="s">
+      <c r="S2" s="17" t="s">
         <v>12</v>
       </c>
-      <c r="T2" s="17"/>
-      <c r="U2" s="17"/>
-      <c r="V2" s="17"/>
-      <c r="W2" s="17"/>
-      <c r="X2" s="17"/>
-      <c r="Y2" s="17"/>
-      <c r="Z2" s="18"/>
+      <c r="T2" s="18"/>
+      <c r="U2" s="18"/>
+      <c r="V2" s="18"/>
+      <c r="W2" s="18"/>
+      <c r="X2" s="18"/>
+      <c r="Y2" s="18"/>
+      <c r="Z2" s="19"/>
     </row>
     <row r="3" spans="1:26">
       <c r="B3" t="s">
@@ -3286,14 +3273,14 @@
       <c r="R3" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="S3" s="16"/>
-      <c r="T3" s="17"/>
-      <c r="U3" s="17"/>
-      <c r="V3" s="17"/>
-      <c r="W3" s="17"/>
-      <c r="X3" s="17"/>
-      <c r="Y3" s="17"/>
-      <c r="Z3" s="18"/>
+      <c r="S3" s="17"/>
+      <c r="T3" s="18"/>
+      <c r="U3" s="18"/>
+      <c r="V3" s="18"/>
+      <c r="W3" s="18"/>
+      <c r="X3" s="18"/>
+      <c r="Y3" s="18"/>
+      <c r="Z3" s="19"/>
     </row>
     <row r="4" spans="1:26">
       <c r="A4">

</xml_diff>